<commit_message>
Nueva rama con pull de direccionar6 en alexCasa1, ahora en nueva rama alexCasa2 apra mantener integro alexCasa1 antes del pull
</commit_message>
<xml_diff>
--- a/servidor/plantillasRegistro/plantillaConfiguracionGeneral.xlsx
+++ b/servidor/plantillasRegistro/plantillaConfiguracionGeneral.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jenny\Desktop\PROYECTOS\ProyectoFulltime\FullTimeActualizado\FulltimeDireccionamiento\FullTime4.0\servidor\plantillasRegistro\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jenny\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5EFB78-B251-4B9B-B984-CA8C32CCDD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9FA9B8-A5F6-4461-997E-B03D1002AE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{384850A9-86C8-4587-9708-E6BD7F8E3DE2}"/>
   </bookViews>
@@ -2668,15 +2668,6 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2693,7 +2684,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5136,7 +5136,7 @@
       <c r="D1" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="22" t="s">
         <v>381</v>
       </c>
     </row>
@@ -8227,24 +8227,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:5" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
     </row>
     <row r="2" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="43" t="s">
         <v>686</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
     </row>
     <row r="3" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="39">
+      <c r="B3" s="36">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="38" t="s">
         <v>695</v>
       </c>
       <c r="D3" s="19"/>
@@ -8253,8 +8253,8 @@
       </c>
     </row>
     <row r="4" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="40"/>
-      <c r="C4" s="42"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="39"/>
       <c r="D4" s="20"/>
       <c r="E4" s="23" t="s">
         <v>687</v>
@@ -8264,188 +8264,193 @@
       <c r="B5" s="16">
         <v>2</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="40" t="s">
         <v>693</v>
       </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
     </row>
     <row r="6" spans="2:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="16">
         <v>3</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="C6" s="41" t="s">
         <v>694</v>
       </c>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
     </row>
     <row r="7" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="38">
+      <c r="B7" s="35">
         <v>4</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="41" t="s">
         <v>688</v>
       </c>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
     </row>
     <row r="8" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="38"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
     </row>
     <row r="9" spans="2:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="28">
         <v>5</v>
       </c>
-      <c r="C9" s="37" t="s">
+      <c r="C9" s="40" t="s">
         <v>689</v>
       </c>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
     </row>
     <row r="10" spans="2:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="16">
         <v>6</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="40" t="s">
         <v>691</v>
       </c>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
     </row>
     <row r="11" spans="2:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="16">
         <v>7</v>
       </c>
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="40" t="s">
         <v>692</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
     </row>
     <row r="12" spans="2:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="27">
         <v>8</v>
       </c>
-      <c r="C12" s="43" t="s">
+      <c r="C12" s="41" t="s">
         <v>690</v>
       </c>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
     </row>
     <row r="13" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="39">
+      <c r="B13" s="36">
         <v>9</v>
       </c>
-      <c r="C13" s="43" t="s">
+      <c r="C13" s="41" t="s">
         <v>696</v>
       </c>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
     </row>
     <row r="14" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="40"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="41"/>
     </row>
     <row r="15" spans="2:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="27">
         <v>10</v>
       </c>
-      <c r="C15" s="43" t="s">
+      <c r="C15" s="41" t="s">
         <v>697</v>
       </c>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
     </row>
     <row r="16" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="38">
+      <c r="B16" s="35">
         <v>11</v>
       </c>
-      <c r="C16" s="43" t="s">
+      <c r="C16" s="41" t="s">
         <v>722</v>
       </c>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
     </row>
     <row r="17" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="38"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
     </row>
     <row r="18" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="38"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
     </row>
     <row r="19" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="38"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="43"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
     </row>
     <row r="20" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="38"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="43"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
     </row>
     <row r="21" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="38"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
     </row>
     <row r="22" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="38"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="43"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
     </row>
     <row r="23" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="38"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="43"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
     </row>
     <row r="24" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="38"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
     </row>
     <row r="25" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="38"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="41"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="41"/>
     </row>
     <row r="26" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="38"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
+      <c r="B26" s="35"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="41"/>
     </row>
     <row r="27" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="38"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="41"/>
     </row>
     <row r="28" spans="2:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="38"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C11:E11"/>
     <mergeCell ref="B16:B28"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
@@ -8458,11 +8463,6 @@
     <mergeCell ref="C16:E28"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="C13:E14"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12727,10 +12727,10 @@
       <c r="Q1" s="21" t="s">
         <v>397</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="21" t="s">
         <v>398</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="21" t="s">
         <v>399</v>
       </c>
       <c r="T1" s="21" t="s">

</xml_diff>